<commit_message>
fix(shearing export): add the missing format when the list overflows the first page
</commit_message>
<xml_diff>
--- a/backend/src/modules/exports/templates/Form 10 - Registro de captura y esquila-v SISTEMA 17ago23.xlsx
+++ b/backend/src/modules/exports/templates/Form 10 - Registro de captura y esquila-v SISTEMA 17ago23.xlsx
@@ -188,11 +188,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="General"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -282,6 +283,13 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -358,7 +366,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -460,6 +468,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1544,91 +1560,91 @@
       <c r="B32" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="C32" s="25" t="n">
+      <c r="C32" s="26" t="n">
         <f aca="false">SUM(C13:C31)</f>
         <v>0</v>
       </c>
-      <c r="D32" s="25" t="n">
+      <c r="D32" s="26" t="n">
         <f aca="false">SUM(D13:D31)</f>
         <v>0</v>
       </c>
-      <c r="E32" s="25" t="n">
+      <c r="E32" s="26" t="n">
         <f aca="false">SUM(E13:E31)</f>
         <v>0</v>
       </c>
-      <c r="F32" s="25" t="n">
+      <c r="F32" s="26" t="n">
         <f aca="false">SUM(F13:F31)</f>
         <v>0</v>
       </c>
-      <c r="G32" s="25" t="n">
+      <c r="G32" s="26" t="n">
         <f aca="false">SUM(G13:G31)</f>
         <v>0</v>
       </c>
-      <c r="H32" s="25" t="n">
+      <c r="H32" s="27" t="n">
         <f aca="false">SUM(H13:H31)</f>
         <v>0</v>
       </c>
-      <c r="I32" s="25" t="n">
+      <c r="I32" s="27" t="n">
         <f aca="false">SUM(I13:I31)</f>
         <v>0</v>
       </c>
-      <c r="J32" s="25" t="n">
+      <c r="J32" s="26" t="n">
         <f aca="false">SUM(J13:J31)</f>
         <v>0</v>
       </c>
-      <c r="K32" s="25" t="n">
+      <c r="K32" s="26" t="n">
         <f aca="false">SUM(K13:K31)</f>
         <v>0</v>
       </c>
-      <c r="L32" s="25" t="n">
+      <c r="L32" s="26" t="n">
         <f aca="false">SUM(L13:L31)</f>
         <v>0</v>
       </c>
-      <c r="M32" s="25" t="n">
+      <c r="M32" s="26" t="n">
         <f aca="false">SUM(M13:M31)</f>
         <v>0</v>
       </c>
-      <c r="N32" s="25" t="n">
+      <c r="N32" s="26" t="n">
         <f aca="false">SUM(N13:N31)</f>
         <v>0</v>
       </c>
-      <c r="O32" s="25" t="n">
+      <c r="O32" s="26" t="n">
         <f aca="false">SUM(O13:O31)</f>
         <v>0</v>
       </c>
-      <c r="P32" s="25" t="n">
+      <c r="P32" s="26" t="n">
         <f aca="false">SUM(P13:P31)</f>
         <v>0</v>
       </c>
-      <c r="Q32" s="25" t="n">
+      <c r="Q32" s="26" t="n">
         <f aca="false">SUM(Q13:Q31)</f>
         <v>0</v>
       </c>
-      <c r="R32" s="25" t="n">
+      <c r="R32" s="26" t="n">
         <f aca="false">SUM(R13:R31)</f>
         <v>0</v>
       </c>
-      <c r="S32" s="25" t="n">
+      <c r="S32" s="26" t="n">
         <f aca="false">SUM(S13:S31)</f>
         <v>0</v>
       </c>
-      <c r="T32" s="25" t="n">
+      <c r="T32" s="26" t="n">
         <f aca="false">SUM(T13:T31)</f>
         <v>0</v>
       </c>
-      <c r="U32" s="25" t="n">
+      <c r="U32" s="26" t="n">
         <f aca="false">SUM(U13:U31)</f>
         <v>0</v>
       </c>
-      <c r="V32" s="25" t="n">
+      <c r="V32" s="26" t="n">
         <f aca="false">SUM(V13:V31)</f>
         <v>0</v>
       </c>
-      <c r="W32" s="25" t="n">
+      <c r="W32" s="26" t="n">
         <f aca="false">SUM(W13:W31)</f>
         <v>0</v>
       </c>
-      <c r="X32" s="25" t="n">
+      <c r="X32" s="26" t="n">
         <f aca="false">SUM(X13:X31)</f>
         <v>0</v>
       </c>

</xml_diff>